<commit_message>
Updated life tables to reflect sex-specific mortality.
Also updated supplemental files to reflect sex differences in outcomes.
</commit_message>
<xml_diff>
--- a/gram_analysis/2025_Jul_paper2_testingstrategies/sim_results/cumulative plots.xlsx
+++ b/gram_analysis/2025_Jul_paper2_testingstrategies/sim_results/cumulative plots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smaya/Documents/GitHub/GRAM/gram_analysis/2025_Jul_paper2_testingstrategies/sim_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F46CCA-1A85-2C4F-B723-2965DD7A82A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E86123-A050-C04B-AD2F-E93B9FA98100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{BACA357A-4B12-A040-BCAB-31D8550BBBCB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
   <si>
     <t>Strategy</t>
   </si>
@@ -94,12 +94,33 @@
   <si>
     <t>Scaling factor</t>
   </si>
+  <si>
+    <t>Consistently Accurate (TP/TN)</t>
+  </si>
+  <si>
+    <t>FP changed to TN</t>
+  </si>
+  <si>
+    <t>FN changed to TP</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>% of Tested</t>
+  </si>
+  <si>
+    <t>% of TP initially missed</t>
+  </si>
+  <si>
+    <t>% of TN initially misclassified</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -117,6 +138,13 @@
     <font>
       <sz val="12"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -143,10 +171,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -162,9 +191,28 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -13772,11 +13820,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{959CE02C-DBC0-6B44-A335-55C332C21024}">
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:AB33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="10" max="10" width="7" customWidth="1"/>
+    <col min="22" max="22" width="37.83203125" customWidth="1"/>
+    <col min="23" max="25" width="13.33203125" customWidth="1"/>
+    <col min="26" max="26" width="13.83203125" customWidth="1"/>
+    <col min="27" max="27" width="13.33203125" customWidth="1"/>
+    <col min="28" max="28" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
@@ -14443,7 +14496,7 @@
       <c r="P16" s="4"/>
       <c r="Q16" s="5"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -14460,7 +14513,7 @@
       <c r="P17" s="4"/>
       <c r="Q17" s="5"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -14470,7 +14523,7 @@
       <c r="G18" s="4"/>
       <c r="H18" s="5"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:28" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -14479,8 +14532,21 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="5"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="X19" s="10"/>
+      <c r="Y19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z19" s="9"/>
+      <c r="AA19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB19" s="9"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -14489,8 +14555,29 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="5"/>
+      <c r="V20" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="W20" t="s">
+        <v>22</v>
+      </c>
+      <c r="X20" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -14499,8 +14586,14 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="5"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="7"/>
+      <c r="X21" s="7"/>
+      <c r="Y21" s="7"/>
+      <c r="Z21" s="7"/>
+      <c r="AA21" s="7"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -14509,8 +14602,32 @@
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="5"/>
+      <c r="V22" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="W22" s="7">
+        <v>8777</v>
+      </c>
+      <c r="X22" s="12">
+        <f>W22/H4</f>
+        <v>0.77419070300785042</v>
+      </c>
+      <c r="Y22" s="7">
+        <v>37</v>
+      </c>
+      <c r="Z22" s="12">
+        <f>Y22 / (F4+Y22)</f>
+        <v>9.3081761006289301E-3</v>
+      </c>
+      <c r="AA22" s="7">
+        <v>382</v>
+      </c>
+      <c r="AB22" s="12">
+        <f>AA22/D4</f>
+        <v>6.9924949661358232E-2</v>
+      </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -14519,8 +14636,32 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="5"/>
+      <c r="V23" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="W23" s="7">
+        <v>23778</v>
+      </c>
+      <c r="X23" s="12">
+        <f t="shared" ref="X23:X32" si="15">W23/H5</f>
+        <v>0.69355967798389917</v>
+      </c>
+      <c r="Y23" s="7">
+        <v>722</v>
+      </c>
+      <c r="Z23" s="12">
+        <f t="shared" ref="Z23:Z24" si="16">Y23 / (F5+Y23)</f>
+        <v>4.5243764882817394E-2</v>
+      </c>
+      <c r="AA23" s="7">
+        <v>3370</v>
+      </c>
+      <c r="AB23" s="12">
+        <f t="shared" ref="AB23:AB32" si="17">AA23/D5</f>
+        <v>0.2479399646851089</v>
+      </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -14529,8 +14670,32 @@
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="5"/>
+      <c r="V24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="W24" s="7">
+        <v>16207</v>
+      </c>
+      <c r="X24" s="12">
+        <f t="shared" si="15"/>
+        <v>0.23075389762938706</v>
+      </c>
+      <c r="Y24" s="7">
+        <v>40850</v>
+      </c>
+      <c r="Z24" s="12">
+        <f t="shared" si="16"/>
+        <v>0.76657471523203669</v>
+      </c>
+      <c r="AA24" s="7">
+        <v>7378</v>
+      </c>
+      <c r="AB24" s="12">
+        <f t="shared" si="17"/>
+        <v>0.36781494590956676</v>
+      </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -14539,8 +14704,194 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
+      <c r="V25" s="7"/>
+      <c r="W25" s="7"/>
+      <c r="X25" s="11"/>
+      <c r="Y25" s="7"/>
+      <c r="Z25" s="12"/>
+      <c r="AA25" s="7"/>
+      <c r="AB25" s="12"/>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V26" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="W26" s="7">
+        <v>9304</v>
+      </c>
+      <c r="X26" s="12">
+        <f t="shared" si="15"/>
+        <v>0.82067566375584367</v>
+      </c>
+      <c r="Y26" s="7">
+        <v>37</v>
+      </c>
+      <c r="Z26" s="12">
+        <f>Y26 / (F8+Y26)</f>
+        <v>9.388480081197666E-3</v>
+      </c>
+      <c r="AA26" s="7">
+        <v>273</v>
+      </c>
+      <c r="AB26" s="12">
+        <f t="shared" si="17"/>
+        <v>4.6555252387448842E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V27" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="W27" s="7">
+        <v>25541</v>
+      </c>
+      <c r="X27" s="12">
+        <f t="shared" si="15"/>
+        <v>0.7449830824874577</v>
+      </c>
+      <c r="Y27" s="7">
+        <v>722</v>
+      </c>
+      <c r="Z27" s="12">
+        <f t="shared" ref="Z27:Z28" si="18">Y27 / (F9+Y27)</f>
+        <v>4.5425946898200578E-2</v>
+      </c>
+      <c r="AA27" s="7">
+        <v>2403</v>
+      </c>
+      <c r="AB27" s="12">
+        <f t="shared" si="17"/>
+        <v>0.16812425662911915</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V28" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="W28" s="7">
+        <v>17731</v>
+      </c>
+      <c r="X28" s="12">
+        <f t="shared" si="15"/>
+        <v>0.25245248095678791</v>
+      </c>
+      <c r="Y28" s="7">
+        <v>40893</v>
+      </c>
+      <c r="Z28" s="12">
+        <f t="shared" si="18"/>
+        <v>0.76614519906323186</v>
+      </c>
+      <c r="AA28" s="7">
+        <v>5468</v>
+      </c>
+      <c r="AB28" s="12">
+        <f t="shared" si="17"/>
+        <v>0.26945252057359681</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V29" s="8"/>
+      <c r="W29" s="7"/>
+      <c r="X29" s="11"/>
+      <c r="Y29" s="7"/>
+      <c r="Z29" s="12"/>
+      <c r="AA29" s="7"/>
+      <c r="AB29" s="12"/>
+    </row>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V30" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="W30" s="7">
+        <v>4265</v>
+      </c>
+      <c r="X30" s="12">
+        <f t="shared" si="15"/>
+        <v>0.40028155795401221</v>
+      </c>
+      <c r="Y30" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="12">
+        <f t="shared" ref="Z23:Z32" si="19">Y30/G12</f>
+        <v>0</v>
+      </c>
+      <c r="AA30" s="7">
+        <v>268</v>
+      </c>
+      <c r="AB30" s="12">
+        <f t="shared" si="17"/>
+        <v>5.5223573047599422E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V31" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="W31" s="7">
+        <v>22361</v>
+      </c>
+      <c r="X31" s="12">
+        <f t="shared" si="15"/>
+        <v>0.75817990709659921</v>
+      </c>
+      <c r="Y31" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="12">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AA31" s="7">
+        <v>1588</v>
+      </c>
+      <c r="AB31" s="12">
+        <f t="shared" si="17"/>
+        <v>0.1628550917854579</v>
+      </c>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V32" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="W32" s="7">
+        <v>8437</v>
+      </c>
+      <c r="X32" s="12">
+        <f t="shared" si="15"/>
+        <v>0.48388391832989219</v>
+      </c>
+      <c r="Y32" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="12">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AA32" s="7">
+        <v>308</v>
+      </c>
+      <c r="AB32" s="12">
+        <f t="shared" si="17"/>
+        <v>0.27402135231316727</v>
+      </c>
+    </row>
+    <row r="33" spans="22:27" x14ac:dyDescent="0.2">
+      <c r="V33" s="7"/>
+      <c r="W33" s="7"/>
+      <c r="X33" s="7"/>
+      <c r="Y33" s="7"/>
+      <c r="Z33" s="7"/>
+      <c r="AA33" s="7"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="V20:V21"/>
+    <mergeCell ref="W19:X19"/>
+    <mergeCell ref="Y19:Z19"/>
+    <mergeCell ref="AA19:AB19"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="H4" formulaRange="1"/>

</xml_diff>